<commit_message>
fix(parity-ingestion): skip Equity Excel footer rows — datetime guard on date column
Replace broken date guard (strptime always returned datetime, so isinstance check
never fired) with a clean isinstance(date_val, datetime) check on the raw openpyxl
cell value. Equity Excel stores real transaction dates as datetime objects; footer
rows (Total Credits, Total Debits, Closing Balance) have None in the date column.
The isinstance check is layout-agnostic and catches every footer variant without
relying on keyword matching.

Update synthetic fixtures and test workbooks to use datetime.datetime objects for
date cells, matching real Equity Bank Excel export behaviour. Rename the embedded-
newline test to reflect the datetime-cell contract now required by the guard.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests_v1/fixtures/test_equity_feb_fixture.xlsx
+++ b/backend/tests_v1/fixtures/test_equity_feb_fixture.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,10 +457,8 @@
           <t>Rent</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>03-02-2025</t>
-        </is>
+      <c r="B2" s="1" t="n">
+        <v>45691</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -481,10 +482,8 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07-02-2025</t>
-        </is>
+      <c r="B3" s="1" t="n">
+        <v>45695</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -508,10 +507,8 @@
           <t>Fee</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10-02-2025</t>
-        </is>
+      <c r="B4" s="1" t="n">
+        <v>45698</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -523,7 +520,6 @@
           <t>55,300.00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -531,10 +527,8 @@
           <t>Refund</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>14-02-2025</t>
-        </is>
+      <c r="B5" s="1" t="n">
+        <v>45702</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -558,10 +552,8 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>18-02-2025</t>
-        </is>
+      <c r="B6" s="1" t="n">
+        <v>45706</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -585,10 +577,8 @@
           <t>Top up</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>21-02-2025</t>
-        </is>
+      <c r="B7" s="1" t="n">
+        <v>45709</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -612,10 +602,8 @@
           <t>Tax</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>25-02-2025</t>
-        </is>
+      <c r="B8" s="1" t="n">
+        <v>45713</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -627,7 +615,6 @@
           <t>62,949.25</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -635,10 +622,8 @@
           <t>Closing</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>28-02-2025</t>
-        </is>
+      <c r="B9" s="1" t="n">
+        <v>45716</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>

</xml_diff>